<commit_message>
updated seabasin to ocean_basin
</commit_message>
<xml_diff>
--- a/data/rawdata.xlsx
+++ b/data/rawdata.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sas21-sem\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86020143-1742-4C2A-8D0D-C6FEEAC52186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D0E0FC-0A31-44D5-B134-3E80A55AB2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-49890" yWindow="-1890" windowWidth="38700" windowHeight="15225" tabRatio="753" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cellcounts" sheetId="1" r:id="rId1"/>
-    <sheet name="seabasin_depth_percentage" sheetId="2" r:id="rId2"/>
+    <sheet name="oceanbasin_depth_percentage" sheetId="2" r:id="rId2"/>
     <sheet name="features" sheetId="9" r:id="rId3"/>
     <sheet name="edx_cell_mol_ratio" sheetId="13" r:id="rId4"/>
     <sheet name="cell_VL" sheetId="24" r:id="rId5"/>
@@ -541,9 +541,6 @@
     <t>filtration</t>
   </si>
   <si>
-    <t>seabasin</t>
-  </si>
-  <si>
     <t>depth_category</t>
   </si>
   <si>
@@ -599,6 +596,9 @@
   </si>
   <si>
     <t>percentage</t>
+  </si>
+  <si>
+    <t>ocean_basin</t>
   </si>
 </sst>
 </file>
@@ -976,19 +976,19 @@
         <v>128</v>
       </c>
       <c r="B1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
-      </c>
-      <c r="D1" t="s">
-        <v>131</v>
       </c>
       <c r="E1" t="s">
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -1025,7 +1025,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F3">
         <v>20</v>
@@ -1125,7 +1125,7 @@
         <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F8">
         <v>2</v>
@@ -1205,7 +1205,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F12">
         <v>7</v>
@@ -1265,7 +1265,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -1345,7 +1345,7 @@
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -1425,7 +1425,7 @@
         <v>6</v>
       </c>
       <c r="E23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -1488,13 +1488,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C1" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="D1" t="s">
         <v>13</v>
@@ -1503,7 +1503,7 @@
         <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1790,7 +1790,7 @@
         <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E15" t="s">
         <v>9</v>
@@ -1811,7 +1811,7 @@
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E16" t="s">
         <v>9</v>
@@ -1832,7 +1832,7 @@
         <v>8</v>
       </c>
       <c r="D17" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E17" t="s">
         <v>9</v>
@@ -1853,7 +1853,7 @@
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E18" t="s">
         <v>9</v>
@@ -1874,7 +1874,7 @@
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -1895,7 +1895,7 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
@@ -1916,7 +1916,7 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
@@ -1937,7 +1937,7 @@
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
@@ -1958,7 +1958,7 @@
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1979,7 +1979,7 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E24" t="s">
         <v>9</v>
@@ -2000,7 +2000,7 @@
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E25" t="s">
         <v>9</v>
@@ -2021,7 +2021,7 @@
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E26" t="s">
         <v>9</v>
@@ -2630,7 +2630,7 @@
         <v>8</v>
       </c>
       <c r="D55" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E55" t="s">
         <v>10</v>
@@ -2651,7 +2651,7 @@
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
@@ -2672,7 +2672,7 @@
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
@@ -2693,7 +2693,7 @@
         <v>2</v>
       </c>
       <c r="D58" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
@@ -2714,7 +2714,7 @@
         <v>2</v>
       </c>
       <c r="D59" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
@@ -2908,22 +2908,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B1" t="s">
         <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -5341,7 +5341,7 @@
         <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C1" t="s">
         <v>21</v>
@@ -7644,13 +7644,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" t="s">
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D1" t="s">
         <v>97</v>
@@ -18783,10 +18783,10 @@
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>138</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>139</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>12</v>
@@ -18807,22 +18807,22 @@
         <v>16</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>142</v>
-      </c>
       <c r="O1" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P1" s="4" t="s">
         <v>97</v>
@@ -22268,7 +22268,7 @@
         <v>9</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G62" s="4" t="s">
         <v>21</v>
@@ -22325,7 +22325,7 @@
         <v>9</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G63" s="4" t="s">
         <v>0</v>
@@ -22382,7 +22382,7 @@
         <v>9</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>62</v>
@@ -22439,7 +22439,7 @@
         <v>9</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G65" s="4" t="s">
         <v>21</v>
@@ -22496,7 +22496,7 @@
         <v>9</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G66" s="4" t="s">
         <v>0</v>
@@ -22553,7 +22553,7 @@
         <v>9</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G67" s="4" t="s">
         <v>62</v>
@@ -22610,7 +22610,7 @@
         <v>9</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G68" s="4" t="s">
         <v>21</v>
@@ -22667,7 +22667,7 @@
         <v>9</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G69" s="4" t="s">
         <v>0</v>
@@ -22724,7 +22724,7 @@
         <v>9</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G70" s="4" t="s">
         <v>62</v>
@@ -22781,7 +22781,7 @@
         <v>9</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G71" s="4" t="s">
         <v>21</v>
@@ -22838,7 +22838,7 @@
         <v>9</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G72" s="4" t="s">
         <v>0</v>
@@ -22895,7 +22895,7 @@
         <v>9</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G73" s="4" t="s">
         <v>62</v>
@@ -22952,7 +22952,7 @@
         <v>9</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G74" s="4" t="s">
         <v>21</v>
@@ -23007,7 +23007,7 @@
         <v>9</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>0</v>
@@ -23064,7 +23064,7 @@
         <v>9</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>62</v>
@@ -23121,7 +23121,7 @@
         <v>9</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G77" s="4" t="s">
         <v>21</v>
@@ -23176,7 +23176,7 @@
         <v>9</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G78" s="4" t="s">
         <v>0</v>
@@ -23233,7 +23233,7 @@
         <v>9</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G79" s="4" t="s">
         <v>62</v>
@@ -23290,7 +23290,7 @@
         <v>9</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G80" s="4" t="s">
         <v>21</v>
@@ -23347,7 +23347,7 @@
         <v>9</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G81" s="4" t="s">
         <v>0</v>
@@ -23404,7 +23404,7 @@
         <v>9</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G82" s="4" t="s">
         <v>62</v>
@@ -23461,7 +23461,7 @@
         <v>9</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G83" s="4" t="s">
         <v>21</v>
@@ -23518,7 +23518,7 @@
         <v>9</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G84" s="4" t="s">
         <v>0</v>
@@ -23575,7 +23575,7 @@
         <v>9</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>62</v>
@@ -23632,7 +23632,7 @@
         <v>9</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G86" s="4" t="s">
         <v>21</v>
@@ -23689,7 +23689,7 @@
         <v>9</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G87" s="4" t="s">
         <v>0</v>
@@ -23746,7 +23746,7 @@
         <v>9</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G88" s="4" t="s">
         <v>62</v>
@@ -23803,7 +23803,7 @@
         <v>9</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>21</v>
@@ -23860,7 +23860,7 @@
         <v>9</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>0</v>
@@ -23917,7 +23917,7 @@
         <v>9</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>62</v>
@@ -23974,7 +23974,7 @@
         <v>9</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G92" s="4" t="s">
         <v>21</v>
@@ -24031,7 +24031,7 @@
         <v>9</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>0</v>
@@ -24088,7 +24088,7 @@
         <v>9</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G94" s="4" t="s">
         <v>62</v>
@@ -24316,7 +24316,7 @@
         <v>9</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G98" s="4" t="s">
         <v>21</v>
@@ -24373,7 +24373,7 @@
         <v>9</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G99" s="4" t="s">
         <v>0</v>
@@ -24430,7 +24430,7 @@
         <v>9</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G100" s="4" t="s">
         <v>62</v>
@@ -24487,7 +24487,7 @@
         <v>9</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>21</v>
@@ -24544,7 +24544,7 @@
         <v>9</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G102" s="4" t="s">
         <v>0</v>
@@ -24601,7 +24601,7 @@
         <v>9</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G103" s="4" t="s">
         <v>62</v>
@@ -26710,7 +26710,7 @@
         <v>10</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G140" s="4" t="s">
         <v>21</v>
@@ -26767,7 +26767,7 @@
         <v>10</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G141" s="4" t="s">
         <v>0</v>
@@ -26824,7 +26824,7 @@
         <v>10</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G142" s="4" t="s">
         <v>62</v>
@@ -26881,7 +26881,7 @@
         <v>10</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>21</v>
@@ -26938,7 +26938,7 @@
         <v>10</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G144" s="4" t="s">
         <v>0</v>
@@ -26995,7 +26995,7 @@
         <v>10</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G145" s="4" t="s">
         <v>62</v>
@@ -28591,7 +28591,7 @@
         <v>9</v>
       </c>
       <c r="F173" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G173" s="4" t="s">
         <v>21</v>
@@ -28648,7 +28648,7 @@
         <v>9</v>
       </c>
       <c r="F174" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G174" s="4" t="s">
         <v>0</v>
@@ -28705,7 +28705,7 @@
         <v>9</v>
       </c>
       <c r="F175" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G175" s="4" t="s">
         <v>62</v>
@@ -28762,7 +28762,7 @@
         <v>9</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G176" s="4" t="s">
         <v>21</v>
@@ -28819,7 +28819,7 @@
         <v>9</v>
       </c>
       <c r="F177" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G177" s="4" t="s">
         <v>0</v>
@@ -28876,7 +28876,7 @@
         <v>9</v>
       </c>
       <c r="F178" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G178" s="4" t="s">
         <v>62</v>
@@ -29617,7 +29617,7 @@
         <v>9</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G191" s="4" t="s">
         <v>21</v>
@@ -29674,7 +29674,7 @@
         <v>9</v>
       </c>
       <c r="F192" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G192" s="4" t="s">
         <v>0</v>
@@ -29731,7 +29731,7 @@
         <v>9</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G193" s="4" t="s">
         <v>62</v>
@@ -29788,7 +29788,7 @@
         <v>9</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G194" s="4" t="s">
         <v>21</v>
@@ -29845,7 +29845,7 @@
         <v>9</v>
       </c>
       <c r="F195" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G195" s="4" t="s">
         <v>0</v>
@@ -29902,7 +29902,7 @@
         <v>9</v>
       </c>
       <c r="F196" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G196" s="4" t="s">
         <v>62</v>
@@ -31327,7 +31327,7 @@
         <v>9</v>
       </c>
       <c r="F221" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G221" s="4" t="s">
         <v>21</v>
@@ -31384,7 +31384,7 @@
         <v>9</v>
       </c>
       <c r="F222" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G222" s="4" t="s">
         <v>0</v>
@@ -31441,7 +31441,7 @@
         <v>9</v>
       </c>
       <c r="F223" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G223" s="4" t="s">
         <v>62</v>
@@ -31498,7 +31498,7 @@
         <v>9</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G224" s="4" t="s">
         <v>21</v>
@@ -31555,7 +31555,7 @@
         <v>9</v>
       </c>
       <c r="F225" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G225" s="4" t="s">
         <v>0</v>
@@ -31612,7 +31612,7 @@
         <v>9</v>
       </c>
       <c r="F226" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G226" s="4" t="s">
         <v>62</v>
@@ -31669,7 +31669,7 @@
         <v>9</v>
       </c>
       <c r="F227" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G227" s="4" t="s">
         <v>21</v>
@@ -31726,7 +31726,7 @@
         <v>9</v>
       </c>
       <c r="F228" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G228" s="4" t="s">
         <v>0</v>
@@ -31783,7 +31783,7 @@
         <v>9</v>
       </c>
       <c r="F229" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G229" s="4" t="s">
         <v>62</v>
@@ -31840,7 +31840,7 @@
         <v>9</v>
       </c>
       <c r="F230" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G230" s="4" t="s">
         <v>21</v>
@@ -31897,7 +31897,7 @@
         <v>9</v>
       </c>
       <c r="F231" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G231" s="4" t="s">
         <v>0</v>
@@ -31954,7 +31954,7 @@
         <v>9</v>
       </c>
       <c r="F232" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G232" s="4" t="s">
         <v>62</v>
@@ -34234,7 +34234,7 @@
         <v>10</v>
       </c>
       <c r="F272" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G272" s="4" t="s">
         <v>21</v>
@@ -34291,7 +34291,7 @@
         <v>10</v>
       </c>
       <c r="F273" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G273" s="4" t="s">
         <v>0</v>
@@ -34348,7 +34348,7 @@
         <v>10</v>
       </c>
       <c r="F274" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G274" s="4" t="s">
         <v>62</v>
@@ -34405,7 +34405,7 @@
         <v>10</v>
       </c>
       <c r="F275" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G275" s="4" t="s">
         <v>21</v>
@@ -34462,7 +34462,7 @@
         <v>10</v>
       </c>
       <c r="F276" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G276" s="4" t="s">
         <v>0</v>
@@ -34519,7 +34519,7 @@
         <v>10</v>
       </c>
       <c r="F277" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G277" s="4" t="s">
         <v>62</v>
@@ -35431,7 +35431,7 @@
         <v>10</v>
       </c>
       <c r="F293" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G293" s="4" t="s">
         <v>21</v>
@@ -35488,7 +35488,7 @@
         <v>10</v>
       </c>
       <c r="F294" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G294" s="4" t="s">
         <v>0</v>
@@ -35545,7 +35545,7 @@
         <v>10</v>
       </c>
       <c r="F295" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G295" s="4" t="s">
         <v>62</v>
@@ -35602,7 +35602,7 @@
         <v>10</v>
       </c>
       <c r="F296" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G296" s="4" t="s">
         <v>21</v>
@@ -35659,7 +35659,7 @@
         <v>10</v>
       </c>
       <c r="F297" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G297" s="4" t="s">
         <v>0</v>
@@ -35716,7 +35716,7 @@
         <v>10</v>
       </c>
       <c r="F298" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G298" s="4" t="s">
         <v>62</v>
@@ -36286,7 +36286,7 @@
         <v>9</v>
       </c>
       <c r="F308" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G308" s="4" t="s">
         <v>21</v>
@@ -36343,7 +36343,7 @@
         <v>9</v>
       </c>
       <c r="F309" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G309" s="4" t="s">
         <v>0</v>
@@ -36400,7 +36400,7 @@
         <v>9</v>
       </c>
       <c r="F310" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G310" s="4" t="s">
         <v>62</v>
@@ -36457,7 +36457,7 @@
         <v>9</v>
       </c>
       <c r="F311" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G311" s="4" t="s">
         <v>21</v>
@@ -36514,7 +36514,7 @@
         <v>9</v>
       </c>
       <c r="F312" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G312" s="4" t="s">
         <v>0</v>
@@ -36571,7 +36571,7 @@
         <v>9</v>
       </c>
       <c r="F313" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G313" s="4" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
updated feature_acronym for morphological features
</commit_message>
<xml_diff>
--- a/data/rawdata.xlsx
+++ b/data/rawdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sas21-sem\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D0E0FC-0A31-44D5-B134-3E80A55AB2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E569A349-5EB7-401E-A875-EB8EA0B23D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-49890" yWindow="-1890" windowWidth="38700" windowHeight="15225" tabRatio="753" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51720" yWindow="-3720" windowWidth="51840" windowHeight="21120" tabRatio="753" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cellcounts" sheetId="1" r:id="rId1"/>
@@ -523,13 +523,7 @@
     <t>Tubules like structures + Vesicle like structures</t>
   </si>
   <si>
-    <t>TL-VL</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Tubules like + Extracellular polymeric substances</t>
-  </si>
-  <si>
-    <t>TL-EPS</t>
   </si>
   <si>
     <t>Pili like structures</t>
@@ -599,6 +593,12 @@
   </si>
   <si>
     <t>ocean_basin</t>
+  </si>
+  <si>
+    <t>TL+ EPS</t>
+  </si>
+  <si>
+    <t>TL+ VL</t>
   </si>
 </sst>
 </file>
@@ -973,22 +973,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" t="s">
         <v>128</v>
-      </c>
-      <c r="B1" t="s">
-        <v>148</v>
-      </c>
-      <c r="C1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D1" t="s">
-        <v>130</v>
       </c>
       <c r="E1" t="s">
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -1025,7 +1025,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F3">
         <v>20</v>
@@ -1125,7 +1125,7 @@
         <v>6</v>
       </c>
       <c r="E8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F8">
         <v>2</v>
@@ -1205,7 +1205,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F12">
         <v>7</v>
@@ -1265,7 +1265,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F15">
         <v>3</v>
@@ -1345,7 +1345,7 @@
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -1425,7 +1425,7 @@
         <v>6</v>
       </c>
       <c r="E23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F23">
         <v>1</v>
@@ -1488,13 +1488,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D1" t="s">
         <v>13</v>
@@ -1503,7 +1503,7 @@
         <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1790,7 +1790,7 @@
         <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E15" t="s">
         <v>9</v>
@@ -1811,7 +1811,7 @@
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E16" t="s">
         <v>9</v>
@@ -1832,7 +1832,7 @@
         <v>8</v>
       </c>
       <c r="D17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E17" t="s">
         <v>9</v>
@@ -1853,7 +1853,7 @@
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
         <v>9</v>
@@ -1874,7 +1874,7 @@
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -1895,7 +1895,7 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
@@ -1916,7 +1916,7 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E21" t="s">
         <v>9</v>
@@ -1937,7 +1937,7 @@
         <v>2</v>
       </c>
       <c r="D22" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
@@ -1958,7 +1958,7 @@
         <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1979,7 +1979,7 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E24" t="s">
         <v>9</v>
@@ -2000,7 +2000,7 @@
         <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E25" t="s">
         <v>9</v>
@@ -2021,7 +2021,7 @@
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E26" t="s">
         <v>9</v>
@@ -2630,7 +2630,7 @@
         <v>8</v>
       </c>
       <c r="D55" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E55" t="s">
         <v>10</v>
@@ -2651,7 +2651,7 @@
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E56" t="s">
         <v>10</v>
@@ -2672,7 +2672,7 @@
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E57" t="s">
         <v>10</v>
@@ -2693,7 +2693,7 @@
         <v>2</v>
       </c>
       <c r="D58" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
@@ -2714,7 +2714,7 @@
         <v>2</v>
       </c>
       <c r="D59" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
@@ -2908,22 +2908,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B1" t="s">
         <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
@@ -3174,10 +3174,10 @@
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E14" t="s">
         <v>1</v>
@@ -3194,10 +3194,10 @@
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E15" t="s">
         <v>95</v>
@@ -3214,10 +3214,10 @@
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D16" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E16" t="s">
         <v>1</v>
@@ -3234,10 +3234,10 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E17" t="s">
         <v>95</v>
@@ -3254,10 +3254,10 @@
         <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D18" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E18" t="s">
         <v>1</v>
@@ -3274,10 +3274,10 @@
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E19" t="s">
         <v>95</v>
@@ -3294,10 +3294,10 @@
         <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E20" t="s">
         <v>1</v>
@@ -3314,10 +3314,10 @@
         <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E21" t="s">
         <v>95</v>
@@ -3334,10 +3334,10 @@
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E22" t="s">
         <v>1</v>
@@ -3354,10 +3354,10 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E23" t="s">
         <v>95</v>
@@ -3374,10 +3374,10 @@
         <v>10</v>
       </c>
       <c r="C24" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D24" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E24" t="s">
         <v>1</v>
@@ -3394,10 +3394,10 @@
         <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D25" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E25" t="s">
         <v>95</v>
@@ -3414,7 +3414,7 @@
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D26" t="s">
         <v>122</v>
@@ -3434,7 +3434,7 @@
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D27" t="s">
         <v>122</v>
@@ -3454,7 +3454,7 @@
         <v>10</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D28" t="s">
         <v>122</v>
@@ -3474,7 +3474,7 @@
         <v>10</v>
       </c>
       <c r="C29" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D29" t="s">
         <v>122</v>
@@ -3494,7 +3494,7 @@
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D30" t="s">
         <v>122</v>
@@ -3514,7 +3514,7 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D31" t="s">
         <v>122</v>
@@ -3534,7 +3534,7 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D32" t="s">
         <v>122</v>
@@ -3554,7 +3554,7 @@
         <v>10</v>
       </c>
       <c r="C33" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D33" t="s">
         <v>122</v>
@@ -3574,7 +3574,7 @@
         <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D34" t="s">
         <v>122</v>
@@ -3594,7 +3594,7 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D35" t="s">
         <v>122</v>
@@ -3614,7 +3614,7 @@
         <v>10</v>
       </c>
       <c r="C36" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D36" t="s">
         <v>122</v>
@@ -3634,7 +3634,7 @@
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D37" t="s">
         <v>122</v>
@@ -4137,7 +4137,7 @@
         <v>108</v>
       </c>
       <c r="D62" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E62" t="s">
         <v>1</v>
@@ -4157,7 +4157,7 @@
         <v>108</v>
       </c>
       <c r="D63" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E63" t="s">
         <v>95</v>
@@ -4177,7 +4177,7 @@
         <v>108</v>
       </c>
       <c r="D64" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E64" t="s">
         <v>1</v>
@@ -4197,7 +4197,7 @@
         <v>108</v>
       </c>
       <c r="D65" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E65" t="s">
         <v>95</v>
@@ -4217,7 +4217,7 @@
         <v>108</v>
       </c>
       <c r="D66" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E66" t="s">
         <v>1</v>
@@ -4237,7 +4237,7 @@
         <v>108</v>
       </c>
       <c r="D67" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E67" t="s">
         <v>95</v>
@@ -4257,7 +4257,7 @@
         <v>108</v>
       </c>
       <c r="D68" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E68" t="s">
         <v>1</v>
@@ -4277,7 +4277,7 @@
         <v>108</v>
       </c>
       <c r="D69" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E69" t="s">
         <v>95</v>
@@ -4297,7 +4297,7 @@
         <v>108</v>
       </c>
       <c r="D70" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E70" t="s">
         <v>1</v>
@@ -4317,7 +4317,7 @@
         <v>108</v>
       </c>
       <c r="D71" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E71" t="s">
         <v>95</v>
@@ -4337,7 +4337,7 @@
         <v>108</v>
       </c>
       <c r="D72" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E72" t="s">
         <v>1</v>
@@ -4357,7 +4357,7 @@
         <v>108</v>
       </c>
       <c r="D73" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E73" t="s">
         <v>95</v>
@@ -5341,7 +5341,7 @@
         <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C1" t="s">
         <v>21</v>
@@ -7644,13 +7644,13 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B1" t="s">
         <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D1" t="s">
         <v>97</v>
@@ -14073,7 +14073,7 @@
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B274" t="s">
         <v>21</v>
@@ -14096,7 +14096,7 @@
     </row>
     <row r="275" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B275" t="s">
         <v>0</v>
@@ -14119,7 +14119,7 @@
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B276" t="s">
         <v>62</v>
@@ -14142,7 +14142,7 @@
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B277" t="s">
         <v>64</v>
@@ -14165,7 +14165,7 @@
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B278" t="s">
         <v>92</v>
@@ -14188,7 +14188,7 @@
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B279" t="s">
         <v>21</v>
@@ -14211,7 +14211,7 @@
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B280" t="s">
         <v>0</v>
@@ -14234,7 +14234,7 @@
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B281" t="s">
         <v>62</v>
@@ -14257,7 +14257,7 @@
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B282" t="s">
         <v>64</v>
@@ -14280,7 +14280,7 @@
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B283" t="s">
         <v>92</v>
@@ -14303,7 +14303,7 @@
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B284" t="s">
         <v>64</v>
@@ -14326,7 +14326,7 @@
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B285" t="s">
         <v>92</v>
@@ -14349,7 +14349,7 @@
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B286" t="s">
         <v>21</v>
@@ -14372,7 +14372,7 @@
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B287" t="s">
         <v>0</v>
@@ -14395,7 +14395,7 @@
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B288" t="s">
         <v>62</v>
@@ -14418,7 +14418,7 @@
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B289" t="s">
         <v>64</v>
@@ -14441,7 +14441,7 @@
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B290" t="s">
         <v>92</v>
@@ -14464,7 +14464,7 @@
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B291" t="s">
         <v>21</v>
@@ -14487,7 +14487,7 @@
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B292" t="s">
         <v>0</v>
@@ -14510,7 +14510,7 @@
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B293" t="s">
         <v>62</v>
@@ -14533,7 +14533,7 @@
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B294" t="s">
         <v>64</v>
@@ -14556,7 +14556,7 @@
     </row>
     <row r="295" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B295" t="s">
         <v>92</v>
@@ -14579,7 +14579,7 @@
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B296" t="s">
         <v>21</v>
@@ -14602,7 +14602,7 @@
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B297" t="s">
         <v>0</v>
@@ -14625,7 +14625,7 @@
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B298" t="s">
         <v>62</v>
@@ -14648,7 +14648,7 @@
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B299" t="s">
         <v>64</v>
@@ -14671,7 +14671,7 @@
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B300" t="s">
         <v>92</v>
@@ -14694,7 +14694,7 @@
     </row>
     <row r="301" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B301" t="s">
         <v>21</v>
@@ -14717,7 +14717,7 @@
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B302" t="s">
         <v>0</v>
@@ -14740,7 +14740,7 @@
     </row>
     <row r="303" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B303" t="s">
         <v>62</v>
@@ -14763,7 +14763,7 @@
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B304" t="s">
         <v>64</v>
@@ -14786,7 +14786,7 @@
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B305" t="s">
         <v>92</v>
@@ -14809,7 +14809,7 @@
     </row>
     <row r="306" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B306" t="s">
         <v>21</v>
@@ -14832,7 +14832,7 @@
     </row>
     <row r="307" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B307" t="s">
         <v>0</v>
@@ -14855,7 +14855,7 @@
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B308" t="s">
         <v>62</v>
@@ -14878,7 +14878,7 @@
     </row>
     <row r="309" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B309" t="s">
         <v>64</v>
@@ -14901,7 +14901,7 @@
     </row>
     <row r="310" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B310" t="s">
         <v>92</v>
@@ -14924,7 +14924,7 @@
     </row>
     <row r="311" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B311" t="s">
         <v>21</v>
@@ -14947,7 +14947,7 @@
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B312" t="s">
         <v>0</v>
@@ -14970,7 +14970,7 @@
     </row>
     <row r="313" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B313" t="s">
         <v>62</v>
@@ -14993,7 +14993,7 @@
     </row>
     <row r="314" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B314" t="s">
         <v>64</v>
@@ -15016,7 +15016,7 @@
     </row>
     <row r="315" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B315" t="s">
         <v>92</v>
@@ -15039,7 +15039,7 @@
     </row>
     <row r="316" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B316" t="s">
         <v>21</v>
@@ -15062,7 +15062,7 @@
     </row>
     <row r="317" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B317" t="s">
         <v>0</v>
@@ -15085,7 +15085,7 @@
     </row>
     <row r="318" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B318" t="s">
         <v>62</v>
@@ -15108,7 +15108,7 @@
     </row>
     <row r="319" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A319" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B319" t="s">
         <v>64</v>
@@ -15131,7 +15131,7 @@
     </row>
     <row r="320" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B320" t="s">
         <v>92</v>
@@ -15154,7 +15154,7 @@
     </row>
     <row r="321" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A321" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B321" t="s">
         <v>21</v>
@@ -15177,7 +15177,7 @@
     </row>
     <row r="322" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A322" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B322" t="s">
         <v>0</v>
@@ -15200,7 +15200,7 @@
     </row>
     <row r="323" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A323" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B323" t="s">
         <v>62</v>
@@ -15223,7 +15223,7 @@
     </row>
     <row r="324" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B324" t="s">
         <v>64</v>
@@ -15246,7 +15246,7 @@
     </row>
     <row r="325" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A325" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B325" t="s">
         <v>92</v>
@@ -15269,7 +15269,7 @@
     </row>
     <row r="326" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A326" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B326" t="s">
         <v>21</v>
@@ -15292,7 +15292,7 @@
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A327" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B327" t="s">
         <v>0</v>
@@ -15315,7 +15315,7 @@
     </row>
     <row r="328" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A328" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B328" t="s">
         <v>62</v>
@@ -15338,7 +15338,7 @@
     </row>
     <row r="329" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A329" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B329" t="s">
         <v>64</v>
@@ -15361,7 +15361,7 @@
     </row>
     <row r="330" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A330" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B330" t="s">
         <v>92</v>
@@ -15384,7 +15384,7 @@
     </row>
     <row r="331" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A331" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B331" t="s">
         <v>21</v>
@@ -15407,7 +15407,7 @@
     </row>
     <row r="332" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A332" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B332" t="s">
         <v>0</v>
@@ -15430,7 +15430,7 @@
     </row>
     <row r="333" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A333" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B333" t="s">
         <v>62</v>
@@ -15453,7 +15453,7 @@
     </row>
     <row r="334" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A334" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B334" t="s">
         <v>64</v>
@@ -15476,7 +15476,7 @@
     </row>
     <row r="335" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A335" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B335" t="s">
         <v>92</v>
@@ -15499,7 +15499,7 @@
     </row>
     <row r="336" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A336" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B336" t="s">
         <v>21</v>
@@ -15522,7 +15522,7 @@
     </row>
     <row r="337" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A337" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B337" t="s">
         <v>0</v>
@@ -15545,7 +15545,7 @@
     </row>
     <row r="338" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A338" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B338" t="s">
         <v>62</v>
@@ -15568,7 +15568,7 @@
     </row>
     <row r="339" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A339" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B339" t="s">
         <v>64</v>
@@ -15591,7 +15591,7 @@
     </row>
     <row r="340" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A340" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B340" t="s">
         <v>92</v>
@@ -15614,7 +15614,7 @@
     </row>
     <row r="341" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A341" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B341" t="s">
         <v>21</v>
@@ -15637,7 +15637,7 @@
     </row>
     <row r="342" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A342" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B342" t="s">
         <v>0</v>
@@ -15660,7 +15660,7 @@
     </row>
     <row r="343" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A343" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B343" t="s">
         <v>62</v>
@@ -15683,7 +15683,7 @@
     </row>
     <row r="344" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A344" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B344" t="s">
         <v>64</v>
@@ -15706,7 +15706,7 @@
     </row>
     <row r="345" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B345" t="s">
         <v>92</v>
@@ -15729,7 +15729,7 @@
     </row>
     <row r="346" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A346" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B346" t="s">
         <v>21</v>
@@ -15752,7 +15752,7 @@
     </row>
     <row r="347" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A347" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B347" t="s">
         <v>0</v>
@@ -15775,7 +15775,7 @@
     </row>
     <row r="348" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B348" t="s">
         <v>62</v>
@@ -15798,7 +15798,7 @@
     </row>
     <row r="349" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A349" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B349" t="s">
         <v>64</v>
@@ -15821,7 +15821,7 @@
     </row>
     <row r="350" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A350" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B350" t="s">
         <v>92</v>
@@ -15844,7 +15844,7 @@
     </row>
     <row r="351" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A351" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B351" t="s">
         <v>21</v>
@@ -15867,7 +15867,7 @@
     </row>
     <row r="352" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A352" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B352" t="s">
         <v>0</v>
@@ -15890,7 +15890,7 @@
     </row>
     <row r="353" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A353" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B353" t="s">
         <v>62</v>
@@ -15913,7 +15913,7 @@
     </row>
     <row r="354" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A354" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B354" t="s">
         <v>64</v>
@@ -15936,7 +15936,7 @@
     </row>
     <row r="355" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A355" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B355" t="s">
         <v>92</v>
@@ -15959,7 +15959,7 @@
     </row>
     <row r="356" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A356" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B356" t="s">
         <v>21</v>
@@ -15982,7 +15982,7 @@
     </row>
     <row r="357" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A357" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B357" t="s">
         <v>0</v>
@@ -16005,7 +16005,7 @@
     </row>
     <row r="358" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A358" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B358" t="s">
         <v>62</v>
@@ -16028,7 +16028,7 @@
     </row>
     <row r="359" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A359" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B359" t="s">
         <v>64</v>
@@ -16051,7 +16051,7 @@
     </row>
     <row r="360" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A360" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B360" t="s">
         <v>92</v>
@@ -16074,7 +16074,7 @@
     </row>
     <row r="361" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A361" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B361" t="s">
         <v>21</v>
@@ -16097,7 +16097,7 @@
     </row>
     <row r="362" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A362" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B362" t="s">
         <v>0</v>
@@ -16120,7 +16120,7 @@
     </row>
     <row r="363" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A363" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B363" t="s">
         <v>62</v>
@@ -16143,7 +16143,7 @@
     </row>
     <row r="364" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A364" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B364" t="s">
         <v>64</v>
@@ -16166,7 +16166,7 @@
     </row>
     <row r="365" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A365" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B365" t="s">
         <v>92</v>
@@ -16189,7 +16189,7 @@
     </row>
     <row r="366" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A366" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B366" t="s">
         <v>21</v>
@@ -16212,7 +16212,7 @@
     </row>
     <row r="367" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A367" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B367" t="s">
         <v>0</v>
@@ -16235,7 +16235,7 @@
     </row>
     <row r="368" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A368" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B368" t="s">
         <v>62</v>
@@ -16258,7 +16258,7 @@
     </row>
     <row r="369" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A369" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B369" t="s">
         <v>64</v>
@@ -16281,7 +16281,7 @@
     </row>
     <row r="370" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A370" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B370" t="s">
         <v>92</v>
@@ -16304,7 +16304,7 @@
     </row>
     <row r="371" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A371" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B371" t="s">
         <v>21</v>
@@ -16327,7 +16327,7 @@
     </row>
     <row r="372" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A372" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B372" t="s">
         <v>0</v>
@@ -16350,7 +16350,7 @@
     </row>
     <row r="373" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A373" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B373" t="s">
         <v>62</v>
@@ -16373,7 +16373,7 @@
     </row>
     <row r="374" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A374" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B374" t="s">
         <v>64</v>
@@ -16396,7 +16396,7 @@
     </row>
     <row r="375" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A375" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B375" t="s">
         <v>92</v>
@@ -16419,7 +16419,7 @@
     </row>
     <row r="376" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A376" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B376" t="s">
         <v>21</v>
@@ -16442,7 +16442,7 @@
     </row>
     <row r="377" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A377" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B377" t="s">
         <v>0</v>
@@ -16465,7 +16465,7 @@
     </row>
     <row r="378" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B378" t="s">
         <v>62</v>
@@ -16488,7 +16488,7 @@
     </row>
     <row r="379" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B379" t="s">
         <v>64</v>
@@ -16511,7 +16511,7 @@
     </row>
     <row r="380" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B380" t="s">
         <v>92</v>
@@ -16534,7 +16534,7 @@
     </row>
     <row r="381" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A381" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B381" t="s">
         <v>21</v>
@@ -16557,7 +16557,7 @@
     </row>
     <row r="382" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A382" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B382" t="s">
         <v>0</v>
@@ -16580,7 +16580,7 @@
     </row>
     <row r="383" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A383" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B383" t="s">
         <v>62</v>
@@ -16603,7 +16603,7 @@
     </row>
     <row r="384" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A384" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B384" t="s">
         <v>64</v>
@@ -16626,7 +16626,7 @@
     </row>
     <row r="385" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A385" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B385" t="s">
         <v>92</v>
@@ -16649,7 +16649,7 @@
     </row>
     <row r="386" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A386" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B386" t="s">
         <v>21</v>
@@ -16672,7 +16672,7 @@
     </row>
     <row r="387" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A387" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B387" t="s">
         <v>0</v>
@@ -16695,7 +16695,7 @@
     </row>
     <row r="388" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A388" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B388" t="s">
         <v>62</v>
@@ -16718,7 +16718,7 @@
     </row>
     <row r="389" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A389" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B389" t="s">
         <v>64</v>
@@ -16741,7 +16741,7 @@
     </row>
     <row r="390" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A390" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B390" t="s">
         <v>92</v>
@@ -16764,7 +16764,7 @@
     </row>
     <row r="391" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A391" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B391" t="s">
         <v>21</v>
@@ -16787,7 +16787,7 @@
     </row>
     <row r="392" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A392" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B392" t="s">
         <v>0</v>
@@ -16810,7 +16810,7 @@
     </row>
     <row r="393" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A393" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B393" t="s">
         <v>62</v>
@@ -16833,7 +16833,7 @@
     </row>
     <row r="394" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A394" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B394" t="s">
         <v>64</v>
@@ -16856,7 +16856,7 @@
     </row>
     <row r="395" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A395" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B395" t="s">
         <v>92</v>
@@ -16879,7 +16879,7 @@
     </row>
     <row r="396" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A396" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B396" t="s">
         <v>21</v>
@@ -16902,7 +16902,7 @@
     </row>
     <row r="397" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A397" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B397" t="s">
         <v>0</v>
@@ -16925,7 +16925,7 @@
     </row>
     <row r="398" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A398" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B398" t="s">
         <v>62</v>
@@ -16948,7 +16948,7 @@
     </row>
     <row r="399" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A399" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B399" t="s">
         <v>64</v>
@@ -16971,7 +16971,7 @@
     </row>
     <row r="400" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A400" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B400" t="s">
         <v>92</v>
@@ -16994,7 +16994,7 @@
     </row>
     <row r="401" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A401" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B401" t="s">
         <v>21</v>
@@ -17017,7 +17017,7 @@
     </row>
     <row r="402" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A402" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B402" t="s">
         <v>0</v>
@@ -17040,7 +17040,7 @@
     </row>
     <row r="403" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A403" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B403" t="s">
         <v>62</v>
@@ -17063,7 +17063,7 @@
     </row>
     <row r="404" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A404" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B404" t="s">
         <v>64</v>
@@ -17086,7 +17086,7 @@
     </row>
     <row r="405" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A405" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B405" t="s">
         <v>92</v>
@@ -17109,7 +17109,7 @@
     </row>
     <row r="406" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A406" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B406" t="s">
         <v>21</v>
@@ -17132,7 +17132,7 @@
     </row>
     <row r="407" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A407" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B407" t="s">
         <v>0</v>
@@ -17155,7 +17155,7 @@
     </row>
     <row r="408" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A408" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B408" t="s">
         <v>62</v>
@@ -17178,7 +17178,7 @@
     </row>
     <row r="409" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A409" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B409" t="s">
         <v>64</v>
@@ -17201,7 +17201,7 @@
     </row>
     <row r="410" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A410" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B410" t="s">
         <v>92</v>
@@ -17224,7 +17224,7 @@
     </row>
     <row r="411" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A411" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B411" t="s">
         <v>21</v>
@@ -17247,7 +17247,7 @@
     </row>
     <row r="412" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A412" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B412" t="s">
         <v>0</v>
@@ -17270,7 +17270,7 @@
     </row>
     <row r="413" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A413" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B413" t="s">
         <v>62</v>
@@ -17293,7 +17293,7 @@
     </row>
     <row r="414" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A414" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B414" t="s">
         <v>64</v>
@@ -17316,7 +17316,7 @@
     </row>
     <row r="415" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A415" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B415" t="s">
         <v>92</v>
@@ -17339,7 +17339,7 @@
     </row>
     <row r="416" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A416" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B416" t="s">
         <v>21</v>
@@ -17362,7 +17362,7 @@
     </row>
     <row r="417" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A417" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B417" t="s">
         <v>0</v>
@@ -17385,7 +17385,7 @@
     </row>
     <row r="418" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A418" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B418" t="s">
         <v>62</v>
@@ -17408,7 +17408,7 @@
     </row>
     <row r="419" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A419" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B419" t="s">
         <v>64</v>
@@ -17431,7 +17431,7 @@
     </row>
     <row r="420" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A420" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B420" t="s">
         <v>92</v>
@@ -17454,7 +17454,7 @@
     </row>
     <row r="421" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A421" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B421" t="s">
         <v>21</v>
@@ -17477,7 +17477,7 @@
     </row>
     <row r="422" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A422" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B422" t="s">
         <v>62</v>
@@ -17500,7 +17500,7 @@
     </row>
     <row r="423" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A423" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B423" t="s">
         <v>64</v>
@@ -17523,7 +17523,7 @@
     </row>
     <row r="424" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B424" t="s">
         <v>92</v>
@@ -17546,7 +17546,7 @@
     </row>
     <row r="425" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A425" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B425" t="s">
         <v>21</v>
@@ -17569,7 +17569,7 @@
     </row>
     <row r="426" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A426" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B426" t="s">
         <v>62</v>
@@ -17592,7 +17592,7 @@
     </row>
     <row r="427" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A427" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B427" t="s">
         <v>64</v>
@@ -17615,7 +17615,7 @@
     </row>
     <row r="428" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A428" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B428" t="s">
         <v>92</v>
@@ -17638,7 +17638,7 @@
     </row>
     <row r="429" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A429" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B429" t="s">
         <v>21</v>
@@ -17661,7 +17661,7 @@
     </row>
     <row r="430" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A430" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B430" t="s">
         <v>62</v>
@@ -17684,7 +17684,7 @@
     </row>
     <row r="431" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A431" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B431" t="s">
         <v>64</v>
@@ -17707,7 +17707,7 @@
     </row>
     <row r="432" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A432" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B432" t="s">
         <v>92</v>
@@ -17730,7 +17730,7 @@
     </row>
     <row r="433" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A433" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B433" t="s">
         <v>21</v>
@@ -17753,7 +17753,7 @@
     </row>
     <row r="434" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A434" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B434" t="s">
         <v>62</v>
@@ -17776,7 +17776,7 @@
     </row>
     <row r="435" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A435" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B435" t="s">
         <v>92</v>
@@ -17799,7 +17799,7 @@
     </row>
     <row r="436" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A436" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B436" t="s">
         <v>21</v>
@@ -17822,7 +17822,7 @@
     </row>
     <row r="437" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A437" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B437" t="s">
         <v>105</v>
@@ -17845,7 +17845,7 @@
     </row>
     <row r="438" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A438" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B438" t="s">
         <v>92</v>
@@ -17868,7 +17868,7 @@
     </row>
     <row r="439" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A439" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B439" t="s">
         <v>21</v>
@@ -17891,7 +17891,7 @@
     </row>
     <row r="440" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A440" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B440" t="s">
         <v>105</v>
@@ -17914,7 +17914,7 @@
     </row>
     <row r="441" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A441" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B441" t="s">
         <v>92</v>
@@ -17937,7 +17937,7 @@
     </row>
     <row r="442" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A442" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B442" t="s">
         <v>21</v>
@@ -17960,7 +17960,7 @@
     </row>
     <row r="443" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A443" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B443" t="s">
         <v>105</v>
@@ -17983,7 +17983,7 @@
     </row>
     <row r="444" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A444" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B444" t="s">
         <v>92</v>
@@ -18006,7 +18006,7 @@
     </row>
     <row r="445" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A445" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B445" t="s">
         <v>21</v>
@@ -18029,7 +18029,7 @@
     </row>
     <row r="446" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A446" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B446" t="s">
         <v>105</v>
@@ -18052,7 +18052,7 @@
     </row>
     <row r="447" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A447" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B447" t="s">
         <v>92</v>
@@ -18075,7 +18075,7 @@
     </row>
     <row r="448" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A448" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B448" t="s">
         <v>21</v>
@@ -18098,7 +18098,7 @@
     </row>
     <row r="449" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A449" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B449" t="s">
         <v>105</v>
@@ -18121,7 +18121,7 @@
     </row>
     <row r="450" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A450" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B450" t="s">
         <v>92</v>
@@ -18144,7 +18144,7 @@
     </row>
     <row r="451" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A451" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B451" t="s">
         <v>21</v>
@@ -18167,7 +18167,7 @@
     </row>
     <row r="452" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A452" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B452" t="s">
         <v>105</v>
@@ -18190,7 +18190,7 @@
     </row>
     <row r="453" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A453" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B453" t="s">
         <v>92</v>
@@ -18213,7 +18213,7 @@
     </row>
     <row r="454" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A454" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B454" t="s">
         <v>21</v>
@@ -18236,7 +18236,7 @@
     </row>
     <row r="455" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A455" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B455" t="s">
         <v>105</v>
@@ -18259,7 +18259,7 @@
     </row>
     <row r="456" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A456" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B456" t="s">
         <v>92</v>
@@ -18282,7 +18282,7 @@
     </row>
     <row r="457" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A457" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B457" t="s">
         <v>21</v>
@@ -18305,7 +18305,7 @@
     </row>
     <row r="458" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A458" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B458" t="s">
         <v>105</v>
@@ -18328,7 +18328,7 @@
     </row>
     <row r="459" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A459" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B459" t="s">
         <v>92</v>
@@ -18351,7 +18351,7 @@
     </row>
     <row r="460" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A460" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B460" t="s">
         <v>21</v>
@@ -18374,7 +18374,7 @@
     </row>
     <row r="461" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A461" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B461" t="s">
         <v>105</v>
@@ -18397,7 +18397,7 @@
     </row>
     <row r="462" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A462" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B462" t="s">
         <v>92</v>
@@ -18420,7 +18420,7 @@
     </row>
     <row r="463" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A463" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B463" t="s">
         <v>21</v>
@@ -18443,7 +18443,7 @@
     </row>
     <row r="464" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A464" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B464" t="s">
         <v>105</v>
@@ -18466,7 +18466,7 @@
     </row>
     <row r="465" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A465" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B465" t="s">
         <v>92</v>
@@ -18489,7 +18489,7 @@
     </row>
     <row r="466" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A466" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B466" t="s">
         <v>21</v>
@@ -18512,7 +18512,7 @@
     </row>
     <row r="467" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A467" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B467" t="s">
         <v>62</v>
@@ -18535,7 +18535,7 @@
     </row>
     <row r="468" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A468" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B468" t="s">
         <v>21</v>
@@ -18558,7 +18558,7 @@
     </row>
     <row r="469" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A469" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B469" t="s">
         <v>62</v>
@@ -18581,7 +18581,7 @@
     </row>
     <row r="470" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A470" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B470" t="s">
         <v>21</v>
@@ -18604,7 +18604,7 @@
     </row>
     <row r="471" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A471" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B471" t="s">
         <v>62</v>
@@ -18627,7 +18627,7 @@
     </row>
     <row r="472" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A472" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B472" t="s">
         <v>21</v>
@@ -18650,7 +18650,7 @@
     </row>
     <row r="473" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A473" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B473" t="s">
         <v>62</v>
@@ -18673,7 +18673,7 @@
     </row>
     <row r="474" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A474" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B474" t="s">
         <v>21</v>
@@ -18696,7 +18696,7 @@
     </row>
     <row r="475" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A475" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B475" t="s">
         <v>62</v>
@@ -18719,7 +18719,7 @@
     </row>
     <row r="476" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A476" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B476" t="s">
         <v>21</v>
@@ -18742,7 +18742,7 @@
     </row>
     <row r="477" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A477" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B477" t="s">
         <v>62</v>
@@ -18783,10 +18783,10 @@
         <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>12</v>
@@ -18807,22 +18807,22 @@
         <v>16</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>17</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="P1" s="4" t="s">
         <v>97</v>
@@ -22268,7 +22268,7 @@
         <v>9</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G62" s="4" t="s">
         <v>21</v>
@@ -22325,7 +22325,7 @@
         <v>9</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G63" s="4" t="s">
         <v>0</v>
@@ -22382,7 +22382,7 @@
         <v>9</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G64" s="4" t="s">
         <v>62</v>
@@ -22439,7 +22439,7 @@
         <v>9</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G65" s="4" t="s">
         <v>21</v>
@@ -22496,7 +22496,7 @@
         <v>9</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G66" s="4" t="s">
         <v>0</v>
@@ -22553,7 +22553,7 @@
         <v>9</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G67" s="4" t="s">
         <v>62</v>
@@ -22610,7 +22610,7 @@
         <v>9</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G68" s="4" t="s">
         <v>21</v>
@@ -22667,7 +22667,7 @@
         <v>9</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G69" s="4" t="s">
         <v>0</v>
@@ -22724,7 +22724,7 @@
         <v>9</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G70" s="4" t="s">
         <v>62</v>
@@ -22781,7 +22781,7 @@
         <v>9</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G71" s="4" t="s">
         <v>21</v>
@@ -22838,7 +22838,7 @@
         <v>9</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G72" s="4" t="s">
         <v>0</v>
@@ -22895,7 +22895,7 @@
         <v>9</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G73" s="4" t="s">
         <v>62</v>
@@ -22952,7 +22952,7 @@
         <v>9</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G74" s="4" t="s">
         <v>21</v>
@@ -23007,7 +23007,7 @@
         <v>9</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G75" s="4" t="s">
         <v>0</v>
@@ -23064,7 +23064,7 @@
         <v>9</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G76" s="4" t="s">
         <v>62</v>
@@ -23121,7 +23121,7 @@
         <v>9</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G77" s="4" t="s">
         <v>21</v>
@@ -23176,7 +23176,7 @@
         <v>9</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G78" s="4" t="s">
         <v>0</v>
@@ -23233,7 +23233,7 @@
         <v>9</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G79" s="4" t="s">
         <v>62</v>
@@ -23290,7 +23290,7 @@
         <v>9</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G80" s="4" t="s">
         <v>21</v>
@@ -23347,7 +23347,7 @@
         <v>9</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G81" s="4" t="s">
         <v>0</v>
@@ -23404,7 +23404,7 @@
         <v>9</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G82" s="4" t="s">
         <v>62</v>
@@ -23461,7 +23461,7 @@
         <v>9</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G83" s="4" t="s">
         <v>21</v>
@@ -23518,7 +23518,7 @@
         <v>9</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G84" s="4" t="s">
         <v>0</v>
@@ -23575,7 +23575,7 @@
         <v>9</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G85" s="4" t="s">
         <v>62</v>
@@ -23632,7 +23632,7 @@
         <v>9</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G86" s="4" t="s">
         <v>21</v>
@@ -23689,7 +23689,7 @@
         <v>9</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G87" s="4" t="s">
         <v>0</v>
@@ -23746,7 +23746,7 @@
         <v>9</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G88" s="4" t="s">
         <v>62</v>
@@ -23803,7 +23803,7 @@
         <v>9</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>21</v>
@@ -23860,7 +23860,7 @@
         <v>9</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>0</v>
@@ -23917,7 +23917,7 @@
         <v>9</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>62</v>
@@ -23974,7 +23974,7 @@
         <v>9</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G92" s="4" t="s">
         <v>21</v>
@@ -24031,7 +24031,7 @@
         <v>9</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G93" s="4" t="s">
         <v>0</v>
@@ -24088,7 +24088,7 @@
         <v>9</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G94" s="4" t="s">
         <v>62</v>
@@ -24316,7 +24316,7 @@
         <v>9</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G98" s="4" t="s">
         <v>21</v>
@@ -24373,7 +24373,7 @@
         <v>9</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G99" s="4" t="s">
         <v>0</v>
@@ -24430,7 +24430,7 @@
         <v>9</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G100" s="4" t="s">
         <v>62</v>
@@ -24487,7 +24487,7 @@
         <v>9</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G101" s="4" t="s">
         <v>21</v>
@@ -24544,7 +24544,7 @@
         <v>9</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G102" s="4" t="s">
         <v>0</v>
@@ -24601,7 +24601,7 @@
         <v>9</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G103" s="4" t="s">
         <v>62</v>
@@ -26710,7 +26710,7 @@
         <v>10</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G140" s="4" t="s">
         <v>21</v>
@@ -26767,7 +26767,7 @@
         <v>10</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G141" s="4" t="s">
         <v>0</v>
@@ -26824,7 +26824,7 @@
         <v>10</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G142" s="4" t="s">
         <v>62</v>
@@ -26881,7 +26881,7 @@
         <v>10</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G143" s="4" t="s">
         <v>21</v>
@@ -26938,7 +26938,7 @@
         <v>10</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G144" s="4" t="s">
         <v>0</v>
@@ -26995,7 +26995,7 @@
         <v>10</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G145" s="4" t="s">
         <v>62</v>
@@ -28591,7 +28591,7 @@
         <v>9</v>
       </c>
       <c r="F173" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G173" s="4" t="s">
         <v>21</v>
@@ -28648,7 +28648,7 @@
         <v>9</v>
       </c>
       <c r="F174" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G174" s="4" t="s">
         <v>0</v>
@@ -28705,7 +28705,7 @@
         <v>9</v>
       </c>
       <c r="F175" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G175" s="4" t="s">
         <v>62</v>
@@ -28762,7 +28762,7 @@
         <v>9</v>
       </c>
       <c r="F176" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G176" s="4" t="s">
         <v>21</v>
@@ -28819,7 +28819,7 @@
         <v>9</v>
       </c>
       <c r="F177" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G177" s="4" t="s">
         <v>0</v>
@@ -28876,7 +28876,7 @@
         <v>9</v>
       </c>
       <c r="F178" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G178" s="4" t="s">
         <v>62</v>
@@ -29617,7 +29617,7 @@
         <v>9</v>
       </c>
       <c r="F191" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G191" s="4" t="s">
         <v>21</v>
@@ -29674,7 +29674,7 @@
         <v>9</v>
       </c>
       <c r="F192" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G192" s="4" t="s">
         <v>0</v>
@@ -29731,7 +29731,7 @@
         <v>9</v>
       </c>
       <c r="F193" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G193" s="4" t="s">
         <v>62</v>
@@ -29788,7 +29788,7 @@
         <v>9</v>
       </c>
       <c r="F194" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G194" s="4" t="s">
         <v>21</v>
@@ -29845,7 +29845,7 @@
         <v>9</v>
       </c>
       <c r="F195" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G195" s="4" t="s">
         <v>0</v>
@@ -29902,7 +29902,7 @@
         <v>9</v>
       </c>
       <c r="F196" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G196" s="4" t="s">
         <v>62</v>
@@ -31327,7 +31327,7 @@
         <v>9</v>
       </c>
       <c r="F221" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G221" s="4" t="s">
         <v>21</v>
@@ -31384,7 +31384,7 @@
         <v>9</v>
       </c>
       <c r="F222" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G222" s="4" t="s">
         <v>0</v>
@@ -31441,7 +31441,7 @@
         <v>9</v>
       </c>
       <c r="F223" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G223" s="4" t="s">
         <v>62</v>
@@ -31498,7 +31498,7 @@
         <v>9</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G224" s="4" t="s">
         <v>21</v>
@@ -31555,7 +31555,7 @@
         <v>9</v>
       </c>
       <c r="F225" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G225" s="4" t="s">
         <v>0</v>
@@ -31612,7 +31612,7 @@
         <v>9</v>
       </c>
       <c r="F226" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G226" s="4" t="s">
         <v>62</v>
@@ -31669,7 +31669,7 @@
         <v>9</v>
       </c>
       <c r="F227" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G227" s="4" t="s">
         <v>21</v>
@@ -31726,7 +31726,7 @@
         <v>9</v>
       </c>
       <c r="F228" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G228" s="4" t="s">
         <v>0</v>
@@ -31783,7 +31783,7 @@
         <v>9</v>
       </c>
       <c r="F229" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G229" s="4" t="s">
         <v>62</v>
@@ -31840,7 +31840,7 @@
         <v>9</v>
       </c>
       <c r="F230" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G230" s="4" t="s">
         <v>21</v>
@@ -31897,7 +31897,7 @@
         <v>9</v>
       </c>
       <c r="F231" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G231" s="4" t="s">
         <v>0</v>
@@ -31954,7 +31954,7 @@
         <v>9</v>
       </c>
       <c r="F232" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G232" s="4" t="s">
         <v>62</v>
@@ -34234,7 +34234,7 @@
         <v>10</v>
       </c>
       <c r="F272" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G272" s="4" t="s">
         <v>21</v>
@@ -34291,7 +34291,7 @@
         <v>10</v>
       </c>
       <c r="F273" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G273" s="4" t="s">
         <v>0</v>
@@ -34348,7 +34348,7 @@
         <v>10</v>
       </c>
       <c r="F274" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G274" s="4" t="s">
         <v>62</v>
@@ -34405,7 +34405,7 @@
         <v>10</v>
       </c>
       <c r="F275" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G275" s="4" t="s">
         <v>21</v>
@@ -34462,7 +34462,7 @@
         <v>10</v>
       </c>
       <c r="F276" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G276" s="4" t="s">
         <v>0</v>
@@ -34519,7 +34519,7 @@
         <v>10</v>
       </c>
       <c r="F277" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G277" s="4" t="s">
         <v>62</v>
@@ -35431,7 +35431,7 @@
         <v>10</v>
       </c>
       <c r="F293" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G293" s="4" t="s">
         <v>21</v>
@@ -35488,7 +35488,7 @@
         <v>10</v>
       </c>
       <c r="F294" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G294" s="4" t="s">
         <v>0</v>
@@ -35545,7 +35545,7 @@
         <v>10</v>
       </c>
       <c r="F295" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G295" s="4" t="s">
         <v>62</v>
@@ -35602,7 +35602,7 @@
         <v>10</v>
       </c>
       <c r="F296" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G296" s="4" t="s">
         <v>21</v>
@@ -35659,7 +35659,7 @@
         <v>10</v>
       </c>
       <c r="F297" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G297" s="4" t="s">
         <v>0</v>
@@ -35716,7 +35716,7 @@
         <v>10</v>
       </c>
       <c r="F298" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G298" s="4" t="s">
         <v>62</v>
@@ -36286,7 +36286,7 @@
         <v>9</v>
       </c>
       <c r="F308" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G308" s="4" t="s">
         <v>21</v>
@@ -36343,7 +36343,7 @@
         <v>9</v>
       </c>
       <c r="F309" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G309" s="4" t="s">
         <v>0</v>
@@ -36400,7 +36400,7 @@
         <v>9</v>
       </c>
       <c r="F310" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G310" s="4" t="s">
         <v>62</v>
@@ -36457,7 +36457,7 @@
         <v>9</v>
       </c>
       <c r="F311" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G311" s="4" t="s">
         <v>21</v>
@@ -36514,7 +36514,7 @@
         <v>9</v>
       </c>
       <c r="F312" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G312" s="4" t="s">
         <v>0</v>
@@ -36571,7 +36571,7 @@
         <v>9</v>
       </c>
       <c r="F313" s="4" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="G313" s="4" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
updated feature_acronym names with spacing issue
</commit_message>
<xml_diff>
--- a/data/rawdata.xlsx
+++ b/data/rawdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sas21-sem\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E569A349-5EB7-401E-A875-EB8EA0B23D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8244284-686F-4FFA-84F1-A7547382B22A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-51720" yWindow="-3720" windowWidth="51840" windowHeight="21120" tabRatio="753" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -595,10 +595,10 @@
     <t>ocean_basin</t>
   </si>
   <si>
-    <t>TL+ EPS</t>
+    <t>TL + EPS</t>
   </si>
   <si>
-    <t>TL+ VL</t>
+    <t>TL + VL</t>
   </si>
 </sst>
 </file>

</xml_diff>